<commit_message>
Dollar to Rupees conversion
</commit_message>
<xml_diff>
--- a/backend/excel/companies.xlsx
+++ b/backend/excel/companies.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -537,6 +537,58 @@
       <c r="N2" t="inlineStr">
         <is>
           <t>2026-10-07 18:58:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>cmp_b7507aded395</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Manufacturing</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>hi@acme.com</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>+1 555 123 4567</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>emp_9370c1d0a3e4</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:59:28</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:59:28</t>
         </is>
       </c>
     </row>

</xml_diff>